<commit_message>
feat(quotations): include Khamis to Muhayil in August Used-Only quotations workbook
</commit_message>
<xml_diff>
--- a/august_import_files/MERCON_August_Quotations_Used_Only.xlsx
+++ b/august_import_files/MERCON_August_Quotations_Used_Only.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="116">
   <si>
     <t>#</t>
   </si>
@@ -85,10 +85,10 @@
     <t>—</t>
   </si>
   <si>
-    <t>Duwadimi</t>
-  </si>
-  <si>
-    <t>RIYADH → Duwadimi</t>
+    <t>DUWADIMI</t>
+  </si>
+  <si>
+    <t>RIYADH → DUWADIMI</t>
   </si>
   <si>
     <t>5 TON</t>
@@ -130,10 +130,10 @@
     <t>JDL | RIYADH SORTING CENTER -&gt; MADINA | 6.5M-10TON</t>
   </si>
   <si>
-    <t>Yanbu</t>
-  </si>
-  <si>
-    <t>RIYADH → Yanbu</t>
+    <t>MADINA</t>
+  </si>
+  <si>
+    <t>RIYADH → MADINA</t>
   </si>
   <si>
     <t>10 TON</t>
@@ -148,10 +148,10 @@
     <t>JEDDAH</t>
   </si>
   <si>
-    <t>Makkah</t>
-  </si>
-  <si>
-    <t>JEDDAH → Makkah</t>
+    <t>MAKKAH</t>
+  </si>
+  <si>
+    <t>JEDDAH → MAKKAH</t>
   </si>
   <si>
     <t>3-4 TON</t>
@@ -163,36 +163,21 @@
     <t>JDL | HAIL SORTING CENTER -&gt; QURAYYAT | 3TON/4TON</t>
   </si>
   <si>
-    <t>Hail</t>
-  </si>
-  <si>
-    <t>Qurayyat</t>
-  </si>
-  <si>
-    <t>Hail → Qurayyat</t>
-  </si>
-  <si>
-    <t>90f8e9c3-70d9-4401-b3a1-325d8c3ff080</t>
+    <t>HAIL</t>
+  </si>
+  <si>
+    <t>QURAYYAT</t>
+  </si>
+  <si>
+    <t>HAIL → QURAYYAT</t>
+  </si>
+  <si>
+    <t>38065f2c-3dd4-43d8-9ee3-4e203e62a42b</t>
   </si>
   <si>
     <t>iMile</t>
   </si>
   <si>
-    <t>iMile | DAMMAM RDC -&gt; JUBAIL | 5M-5TON</t>
-  </si>
-  <si>
-    <t>DAMMAM RDC</t>
-  </si>
-  <si>
-    <t>JUBAIL</t>
-  </si>
-  <si>
-    <t>DAMMAM RDC → JUBAIL</t>
-  </si>
-  <si>
-    <t>38065f2c-3dd4-43d8-9ee3-4e203e62a42b</t>
-  </si>
-  <si>
     <t>iMile | INSIDE RIYADH -&gt; INSIDE RIYADH | 6.5M-10TON</t>
   </si>
   <si>
@@ -208,34 +193,67 @@
     <t>iMile | INSIDE RIYADH -&gt; INSIDE RIYADH | 13.5M-20TON</t>
   </si>
   <si>
-    <t>239d2a77-6e3d-42da-9bfc-db8dac32ed06</t>
-  </si>
-  <si>
-    <t>iMile | KHAMIS MUSHAIT DISTIBUTION CENTRE -&gt; JAZAN STATION | 13.5M-20TON</t>
+    <t>e66e9210-f4a6-463b-80c6-a292aad63e55</t>
+  </si>
+  <si>
+    <t>iMile | KHAMIS MUSHAIT DISTIBUTION CENTRE -&gt; ABHA STATION | 6.5M-10TON</t>
   </si>
   <si>
     <t>KHAMIS MUSHAIT DISTIBUTION CENTRE</t>
   </si>
   <si>
-    <t>JAZAN</t>
-  </si>
-  <si>
-    <t>KHAMIS MUSHAIT DISTIBUTION CENTRE → JAZAN</t>
-  </si>
-  <si>
-    <t>a158a42b-d5e8-49b0-a02a-cd47b8b51c29</t>
-  </si>
-  <si>
-    <t>iMile | RIYADH CENTRE -&gt; BURAIDAH STATION | 6.5M-10TON</t>
+    <t>ABHA</t>
+  </si>
+  <si>
+    <t>KHAMIS MUSHAIT DISTIBUTION CENTRE → ABHA</t>
+  </si>
+  <si>
+    <t>f43d1d95-570c-477f-b5c5-682a6f974f82</t>
+  </si>
+  <si>
+    <t>iMile | RIYADH CENTRE -&gt; DUWADIMI STATION | 6.5M-10TON</t>
   </si>
   <si>
     <t>RIYADH CENTRE</t>
   </si>
   <si>
-    <t>Buraidah</t>
-  </si>
-  <si>
-    <t>RIYADH CENTRE → Buraidah</t>
+    <t>RIYADH CENTRE → DUWADIMI</t>
+  </si>
+  <si>
+    <t>4197a83a-2e36-45ed-a0f4-8da44b2e59d7</t>
+  </si>
+  <si>
+    <t>iMile | KHAMIS MUSHAIT DISTRIBUTION CENTRE -&gt; MUHAYIL STATION | 6.5M-10TON</t>
+  </si>
+  <si>
+    <t>KHAMIS MUSHAIT DISTRIBUTION CENTRE</t>
+  </si>
+  <si>
+    <t>MUHAYIL</t>
+  </si>
+  <si>
+    <t>KHAMIS MUSHAIT DISTRIBUTION CENTRE → MUHAYIL</t>
+  </si>
+  <si>
+    <t>SINGLE_TRIP</t>
+  </si>
+  <si>
+    <t>MONTHLY</t>
+  </si>
+  <si>
+    <t>61c3ba0d-9bbc-4198-aba9-ba57cc25d5af</t>
+  </si>
+  <si>
+    <t>iMile | RIYADH DISTRIBUTION CENTRE -&gt; AL BAHAH STATION | 6.5M-10TON</t>
+  </si>
+  <si>
+    <t>AL</t>
+  </si>
+  <si>
+    <t>AL BAHAH STATION</t>
+  </si>
+  <si>
+    <t>RIYADH CENTRE → AL → AL BAHAH STATION</t>
   </si>
   <si>
     <t>a51615b5-9ae7-4151-a854-a6972605499d</t>
@@ -247,15 +265,9 @@
     <t>Shipa | RIYADH -&gt; MAKKAH | 5 TON</t>
   </si>
   <si>
-    <t>MAKKAH</t>
-  </si>
-  <si>
     <t>RIYADH → MAKKAH</t>
   </si>
   <si>
-    <t>SINGLE_TRIP</t>
-  </si>
-  <si>
     <t>3ca8e844-de94-4f91-aa46-27d9b509e456</t>
   </si>
   <si>
@@ -289,16 +301,13 @@
     <t>Shipa | RUH -&gt; JED | 5 TON</t>
   </si>
   <si>
-    <t>Riyadh</t>
-  </si>
-  <si>
-    <t>Jeddah</t>
-  </si>
-  <si>
-    <t>Riyadh → Jeddah</t>
-  </si>
-  <si>
-    <t>MONTHLY</t>
+    <t>RUH</t>
+  </si>
+  <si>
+    <t>JED</t>
+  </si>
+  <si>
+    <t>RUH → JED</t>
   </si>
   <si>
     <t>53e8f892-b5b2-499e-a4ff-737a528253d8</t>
@@ -310,10 +319,10 @@
     <t>AKS | RIYADH -&gt; UNAIZA | LORRY</t>
   </si>
   <si>
-    <t>Unaizah</t>
-  </si>
-  <si>
-    <t>RIYADH → Unaizah</t>
+    <t>UNAIZA</t>
+  </si>
+  <si>
+    <t>RIYADH → UNAIZA</t>
   </si>
   <si>
     <t>5eb9343b-23ae-4abf-b206-430a40ccdcc8</t>
@@ -350,25 +359,13 @@
   </si>
   <si>
     <t>[HISTORICAL] iMile | RIYADH CENTRE -&gt; AL BAHAH STATION | 6.5M-10TON</t>
-  </si>
-  <si>
-    <t>AL</t>
-  </si>
-  <si>
-    <t>AL BAHAH STATION</t>
-  </si>
-  <si>
-    <t>RIYADH CENTRE → AL → AL BAHAH STATION</t>
-  </si>
-  <si>
-    <t>Inactive</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -378,10 +375,8 @@
     </font>
     <font>
       <b/>
-    </font>
-    <font>
-      <b/>
       <color rgb="FFFFFF"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="3">
@@ -393,7 +388,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FA634E"/>
+        <fgColor rgb="3E3C3D"/>
       </patternFill>
     </fill>
   </fills>
@@ -409,10 +404,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -752,85 +748,85 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:S20"/>
+  <dimension ref="A1:S21"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="15" customWidth="1"/>
-    <col min="2" max="2" width="39" customWidth="1"/>
-    <col min="3" max="3" width="16" customWidth="1"/>
-    <col min="4" max="4" width="55" customWidth="1"/>
-    <col min="5" max="5" width="36" customWidth="1"/>
-    <col min="6" max="6" width="16" customWidth="1"/>
-    <col min="7" max="8" width="22" customWidth="1"/>
-    <col min="9" max="9" width="55" customWidth="1"/>
-    <col min="10" max="10" width="15" customWidth="1"/>
-    <col min="11" max="11" width="16" customWidth="1"/>
-    <col min="12" max="12" width="15" customWidth="1"/>
-    <col min="13" max="13" width="17" customWidth="1"/>
-    <col min="14" max="14" width="21" customWidth="1"/>
-    <col min="15" max="15" width="22" customWidth="1"/>
-    <col min="16" max="16" width="24" customWidth="1"/>
-    <col min="17" max="17" width="29" customWidth="1"/>
-    <col min="18" max="18" width="33" customWidth="1"/>
-    <col min="19" max="19" width="15" customWidth="1"/>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="2" width="40" customWidth="1"/>
+    <col min="3" max="3" width="17" customWidth="1"/>
+    <col min="4" max="4" width="50" customWidth="1"/>
+    <col min="5" max="5" width="38" customWidth="1"/>
+    <col min="6" max="6" width="17" customWidth="1"/>
+    <col min="7" max="8" width="23" customWidth="1"/>
+    <col min="9" max="9" width="50" customWidth="1"/>
+    <col min="10" max="10" width="16" customWidth="1"/>
+    <col min="11" max="11" width="17" customWidth="1"/>
+    <col min="12" max="12" width="16" customWidth="1"/>
+    <col min="13" max="13" width="18" customWidth="1"/>
+    <col min="14" max="14" width="22" customWidth="1"/>
+    <col min="15" max="15" width="23" customWidth="1"/>
+    <col min="16" max="16" width="25" customWidth="1"/>
+    <col min="17" max="17" width="30" customWidth="1"/>
+    <col min="18" max="18" width="34" customWidth="1"/>
+    <col min="19" max="19" width="16" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="2" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
     </row>
@@ -1146,22 +1142,22 @@
         <v>56</v>
       </c>
       <c r="F7" t="s">
-        <v>23</v>
+        <v>56</v>
       </c>
       <c r="G7" t="s">
         <v>23</v>
       </c>
       <c r="H7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I7" t="s">
         <v>57</v>
       </c>
-      <c r="I7" t="s">
-        <v>58</v>
-      </c>
       <c r="J7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K7" t="s">
-        <v>26</v>
+        <v>41</v>
       </c>
       <c r="L7" t="s">
         <v>27</v>
@@ -1170,19 +1166,19 @@
         <v>28</v>
       </c>
       <c r="N7">
-        <v>499</v>
+        <v>545</v>
       </c>
       <c r="O7">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="P7">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="Q7">
-        <v>10978</v>
+        <v>5450</v>
       </c>
       <c r="R7">
-        <v>1100</v>
+        <v>600</v>
       </c>
       <c r="S7" t="s">
         <v>29</v>
@@ -1193,19 +1189,19 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C8" t="s">
         <v>54</v>
       </c>
       <c r="D8" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E8" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="F8" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="G8" t="s">
         <v>23</v>
@@ -1214,13 +1210,13 @@
         <v>22</v>
       </c>
       <c r="I8" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="J8">
         <v>3</v>
       </c>
       <c r="K8" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="L8" t="s">
         <v>27</v>
@@ -1229,19 +1225,19 @@
         <v>28</v>
       </c>
       <c r="N8">
-        <v>545</v>
+        <v>1050</v>
       </c>
       <c r="O8">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="P8">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="Q8">
-        <v>5450</v>
+        <v>2100</v>
       </c>
       <c r="R8">
-        <v>600</v>
+        <v>128</v>
       </c>
       <c r="S8" t="s">
         <v>29</v>
@@ -1252,34 +1248,34 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="C9" t="s">
         <v>54</v>
       </c>
       <c r="D9" t="s">
+        <v>61</v>
+      </c>
+      <c r="E9" t="s">
+        <v>62</v>
+      </c>
+      <c r="F9" t="s">
+        <v>23</v>
+      </c>
+      <c r="G9" t="s">
+        <v>23</v>
+      </c>
+      <c r="H9" t="s">
+        <v>63</v>
+      </c>
+      <c r="I9" t="s">
         <v>64</v>
       </c>
-      <c r="E9" t="s">
-        <v>61</v>
-      </c>
-      <c r="F9" t="s">
-        <v>61</v>
-      </c>
-      <c r="G9" t="s">
-        <v>23</v>
-      </c>
-      <c r="H9" t="s">
-        <v>22</v>
-      </c>
-      <c r="I9" t="s">
-        <v>62</v>
-      </c>
       <c r="J9">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K9" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="L9" t="s">
         <v>27</v>
@@ -1288,19 +1284,19 @@
         <v>28</v>
       </c>
       <c r="N9">
-        <v>1050</v>
+        <v>624</v>
       </c>
       <c r="O9">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="P9">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="Q9">
-        <v>2100</v>
+        <v>13728</v>
       </c>
       <c r="R9">
-        <v>128</v>
+        <v>1320</v>
       </c>
       <c r="S9" t="s">
         <v>29</v>
@@ -1329,16 +1325,16 @@
         <v>23</v>
       </c>
       <c r="H10" t="s">
+        <v>24</v>
+      </c>
+      <c r="I10" t="s">
         <v>68</v>
-      </c>
-      <c r="I10" t="s">
-        <v>69</v>
       </c>
       <c r="J10">
         <v>2</v>
       </c>
       <c r="K10" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="L10" t="s">
         <v>27</v>
@@ -1347,19 +1343,19 @@
         <v>28</v>
       </c>
       <c r="N10">
-        <v>1750</v>
+        <v>1015</v>
       </c>
       <c r="O10">
-        <v>149</v>
+        <v>64</v>
       </c>
       <c r="P10">
-        <v>22</v>
+        <v>4</v>
       </c>
       <c r="Q10">
-        <v>38500</v>
+        <v>4060</v>
       </c>
       <c r="R10">
-        <v>3278</v>
+        <v>256</v>
       </c>
       <c r="S10" t="s">
         <v>29</v>
@@ -1370,28 +1366,28 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C11" t="s">
         <v>54</v>
       </c>
       <c r="D11" t="s">
+        <v>70</v>
+      </c>
+      <c r="E11" t="s">
         <v>71</v>
       </c>
-      <c r="E11" t="s">
+      <c r="F11" t="s">
+        <v>23</v>
+      </c>
+      <c r="G11" t="s">
+        <v>23</v>
+      </c>
+      <c r="H11" t="s">
         <v>72</v>
       </c>
-      <c r="F11" t="s">
-        <v>23</v>
-      </c>
-      <c r="G11" t="s">
-        <v>23</v>
-      </c>
-      <c r="H11" t="s">
+      <c r="I11" t="s">
         <v>73</v>
-      </c>
-      <c r="I11" t="s">
-        <v>74</v>
       </c>
       <c r="J11">
         <v>2</v>
@@ -1400,25 +1396,25 @@
         <v>41</v>
       </c>
       <c r="L11" t="s">
-        <v>27</v>
+        <v>74</v>
       </c>
       <c r="M11" t="s">
-        <v>28</v>
+        <v>75</v>
       </c>
       <c r="N11">
-        <v>1015</v>
+        <v>499</v>
       </c>
       <c r="O11">
-        <v>64</v>
+        <v>50</v>
       </c>
       <c r="P11">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="Q11">
-        <v>4060</v>
+        <v>10978</v>
       </c>
       <c r="R11">
-        <v>256</v>
+        <v>1100</v>
       </c>
       <c r="S11" t="s">
         <v>29</v>
@@ -1429,55 +1425,55 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C12" t="s">
-        <v>76</v>
+        <v>54</v>
       </c>
       <c r="D12" t="s">
         <v>77</v>
       </c>
       <c r="E12" t="s">
+        <v>67</v>
+      </c>
+      <c r="F12" t="s">
+        <v>78</v>
+      </c>
+      <c r="G12" t="s">
+        <v>23</v>
+      </c>
+      <c r="H12" t="s">
+        <v>79</v>
+      </c>
+      <c r="I12" t="s">
+        <v>80</v>
+      </c>
+      <c r="J12">
+        <v>3</v>
+      </c>
+      <c r="K12" t="s">
+        <v>41</v>
+      </c>
+      <c r="L12" t="s">
+        <v>74</v>
+      </c>
+      <c r="M12" t="s">
+        <v>75</v>
+      </c>
+      <c r="N12">
+        <v>1750</v>
+      </c>
+      <c r="O12">
+        <v>149</v>
+      </c>
+      <c r="P12">
         <v>22</v>
       </c>
-      <c r="F12" t="s">
-        <v>23</v>
-      </c>
-      <c r="G12" t="s">
-        <v>23</v>
-      </c>
-      <c r="H12" t="s">
-        <v>78</v>
-      </c>
-      <c r="I12" t="s">
-        <v>79</v>
-      </c>
-      <c r="J12">
-        <v>2</v>
-      </c>
-      <c r="K12" t="s">
-        <v>26</v>
-      </c>
-      <c r="L12" t="s">
-        <v>80</v>
-      </c>
-      <c r="M12" t="s">
-        <v>28</v>
-      </c>
-      <c r="N12">
-        <v>1375</v>
-      </c>
-      <c r="O12">
-        <v>1200</v>
-      </c>
-      <c r="P12">
-        <v>4</v>
-      </c>
       <c r="Q12">
-        <v>5500</v>
+        <v>38500</v>
       </c>
       <c r="R12">
-        <v>4800</v>
+        <v>3278</v>
       </c>
       <c r="S12" t="s">
         <v>29</v>
@@ -1491,52 +1487,52 @@
         <v>81</v>
       </c>
       <c r="C13" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="D13" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="E13" t="s">
-        <v>83</v>
+        <v>22</v>
       </c>
       <c r="F13" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G13" t="s">
         <v>23</v>
       </c>
       <c r="H13" t="s">
+        <v>45</v>
+      </c>
+      <c r="I13" t="s">
         <v>84</v>
       </c>
-      <c r="I13" t="s">
-        <v>85</v>
-      </c>
       <c r="J13">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K13" t="s">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="L13" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="M13" t="s">
         <v>28</v>
       </c>
       <c r="N13">
-        <v>500</v>
+        <v>1375</v>
       </c>
       <c r="O13">
-        <v>45</v>
+        <v>1200</v>
       </c>
       <c r="P13">
         <v>4</v>
       </c>
       <c r="Q13">
-        <v>2000</v>
+        <v>5500</v>
       </c>
       <c r="R13">
-        <v>180</v>
+        <v>4800</v>
       </c>
       <c r="S13" t="s">
         <v>29</v>
@@ -1547,25 +1543,25 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
+        <v>85</v>
+      </c>
+      <c r="C14" t="s">
+        <v>82</v>
+      </c>
+      <c r="D14" t="s">
         <v>86</v>
       </c>
-      <c r="C14" t="s">
-        <v>76</v>
-      </c>
-      <c r="D14" t="s">
+      <c r="E14" t="s">
         <v>87</v>
       </c>
-      <c r="E14" t="s">
+      <c r="F14" t="s">
         <v>22</v>
       </c>
-      <c r="F14" t="s">
+      <c r="G14" t="s">
+        <v>23</v>
+      </c>
+      <c r="H14" t="s">
         <v>88</v>
-      </c>
-      <c r="G14" t="s">
-        <v>23</v>
-      </c>
-      <c r="H14" t="s">
-        <v>78</v>
       </c>
       <c r="I14" t="s">
         <v>89</v>
@@ -1574,28 +1570,28 @@
         <v>3</v>
       </c>
       <c r="K14" t="s">
-        <v>26</v>
+        <v>41</v>
       </c>
       <c r="L14" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="M14" t="s">
         <v>28</v>
       </c>
       <c r="N14">
-        <v>1500</v>
+        <v>500</v>
       </c>
       <c r="O14">
-        <v>149</v>
+        <v>45</v>
       </c>
       <c r="P14">
-        <v>22</v>
+        <v>4</v>
       </c>
       <c r="Q14">
-        <v>33000</v>
+        <v>2000</v>
       </c>
       <c r="R14">
-        <v>3278</v>
+        <v>180</v>
       </c>
       <c r="S14" t="s">
         <v>29</v>
@@ -1609,52 +1605,52 @@
         <v>90</v>
       </c>
       <c r="C15" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="D15" t="s">
         <v>91</v>
       </c>
       <c r="E15" t="s">
+        <v>22</v>
+      </c>
+      <c r="F15" t="s">
         <v>92</v>
       </c>
-      <c r="F15" t="s">
-        <v>23</v>
-      </c>
       <c r="G15" t="s">
         <v>23</v>
       </c>
       <c r="H15" t="s">
+        <v>45</v>
+      </c>
+      <c r="I15" t="s">
         <v>93</v>
       </c>
-      <c r="I15" t="s">
-        <v>94</v>
-      </c>
       <c r="J15">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K15" t="s">
         <v>26</v>
       </c>
       <c r="L15" t="s">
-        <v>27</v>
+        <v>74</v>
       </c>
       <c r="M15" t="s">
-        <v>95</v>
+        <v>28</v>
       </c>
       <c r="N15">
-        <v>49850</v>
+        <v>1500</v>
       </c>
       <c r="O15">
         <v>149</v>
       </c>
       <c r="P15">
-        <v>44</v>
+        <v>22</v>
       </c>
       <c r="Q15">
-        <v>2193400</v>
+        <v>33000</v>
       </c>
       <c r="R15">
-        <v>6556</v>
+        <v>3278</v>
       </c>
       <c r="S15" t="s">
         <v>29</v>
@@ -1665,55 +1661,55 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
+        <v>94</v>
+      </c>
+      <c r="C16" t="s">
+        <v>82</v>
+      </c>
+      <c r="D16" t="s">
+        <v>95</v>
+      </c>
+      <c r="E16" t="s">
         <v>96</v>
       </c>
-      <c r="C16" t="s">
+      <c r="F16" t="s">
+        <v>23</v>
+      </c>
+      <c r="G16" t="s">
+        <v>23</v>
+      </c>
+      <c r="H16" t="s">
         <v>97</v>
       </c>
-      <c r="D16" t="s">
+      <c r="I16" t="s">
         <v>98</v>
-      </c>
-      <c r="E16" t="s">
-        <v>22</v>
-      </c>
-      <c r="F16" t="s">
-        <v>23</v>
-      </c>
-      <c r="G16" t="s">
-        <v>23</v>
-      </c>
-      <c r="H16" t="s">
-        <v>99</v>
-      </c>
-      <c r="I16" t="s">
-        <v>100</v>
       </c>
       <c r="J16">
         <v>2</v>
       </c>
       <c r="K16" t="s">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="L16" t="s">
-        <v>80</v>
+        <v>27</v>
       </c>
       <c r="M16" t="s">
-        <v>28</v>
+        <v>75</v>
       </c>
       <c r="N16">
-        <v>1300</v>
+        <v>49850</v>
       </c>
       <c r="O16">
-        <v>1650</v>
+        <v>149</v>
       </c>
       <c r="P16">
-        <v>2</v>
+        <v>44</v>
       </c>
       <c r="Q16">
-        <v>2600</v>
+        <v>2193400</v>
       </c>
       <c r="R16">
-        <v>3300</v>
+        <v>6556</v>
       </c>
       <c r="S16" t="s">
         <v>29</v>
@@ -1724,13 +1720,13 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
+        <v>99</v>
+      </c>
+      <c r="C17" t="s">
+        <v>100</v>
+      </c>
+      <c r="D17" t="s">
         <v>101</v>
-      </c>
-      <c r="C17" t="s">
-        <v>97</v>
-      </c>
-      <c r="D17" t="s">
-        <v>102</v>
       </c>
       <c r="E17" t="s">
         <v>22</v>
@@ -1742,7 +1738,7 @@
         <v>23</v>
       </c>
       <c r="H17" t="s">
-        <v>84</v>
+        <v>102</v>
       </c>
       <c r="I17" t="s">
         <v>103</v>
@@ -1754,25 +1750,25 @@
         <v>41</v>
       </c>
       <c r="L17" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="M17" t="s">
         <v>28</v>
       </c>
       <c r="N17">
-        <v>450</v>
+        <v>1300</v>
       </c>
       <c r="O17">
-        <v>185</v>
+        <v>1650</v>
       </c>
       <c r="P17">
         <v>2</v>
       </c>
       <c r="Q17">
-        <v>900</v>
+        <v>2600</v>
       </c>
       <c r="R17">
-        <v>370</v>
+        <v>3300</v>
       </c>
       <c r="S17" t="s">
         <v>29</v>
@@ -1786,7 +1782,7 @@
         <v>104</v>
       </c>
       <c r="C18" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="D18" t="s">
         <v>105</v>
@@ -1801,37 +1797,37 @@
         <v>23</v>
       </c>
       <c r="H18" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="I18" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="J18">
         <v>2</v>
       </c>
       <c r="K18" t="s">
-        <v>106</v>
+        <v>41</v>
       </c>
       <c r="L18" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="M18" t="s">
         <v>28</v>
       </c>
       <c r="N18">
+        <v>450</v>
+      </c>
+      <c r="O18">
+        <v>185</v>
+      </c>
+      <c r="P18">
+        <v>2</v>
+      </c>
+      <c r="Q18">
         <v>900</v>
       </c>
-      <c r="O18">
-        <v>1250</v>
-      </c>
-      <c r="P18">
-        <v>4</v>
-      </c>
-      <c r="Q18">
-        <v>3600</v>
-      </c>
       <c r="R18">
-        <v>5000</v>
+        <v>370</v>
       </c>
       <c r="S18" t="s">
         <v>29</v>
@@ -1845,7 +1841,7 @@
         <v>107</v>
       </c>
       <c r="C19" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="D19" t="s">
         <v>108</v>
@@ -1860,37 +1856,37 @@
         <v>23</v>
       </c>
       <c r="H19" t="s">
-        <v>109</v>
+        <v>88</v>
       </c>
       <c r="I19" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="J19">
         <v>2</v>
       </c>
       <c r="K19" t="s">
-        <v>47</v>
+        <v>109</v>
       </c>
       <c r="L19" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="M19" t="s">
         <v>28</v>
       </c>
       <c r="N19">
-        <v>850</v>
+        <v>900</v>
       </c>
       <c r="O19">
-        <v>124</v>
+        <v>1250</v>
       </c>
       <c r="P19">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="Q19">
-        <v>5100</v>
+        <v>3600</v>
       </c>
       <c r="R19">
-        <v>744</v>
+        <v>5000</v>
       </c>
       <c r="S19" t="s">
         <v>29</v>
@@ -1901,58 +1897,117 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
+        <v>110</v>
+      </c>
+      <c r="C20" t="s">
+        <v>100</v>
+      </c>
+      <c r="D20" t="s">
         <v>111</v>
       </c>
-      <c r="C20" t="s">
-        <v>54</v>
-      </c>
-      <c r="D20" t="s">
+      <c r="E20" t="s">
+        <v>22</v>
+      </c>
+      <c r="F20" t="s">
+        <v>23</v>
+      </c>
+      <c r="G20" t="s">
+        <v>23</v>
+      </c>
+      <c r="H20" t="s">
         <v>112</v>
       </c>
-      <c r="E20" t="s">
-        <v>72</v>
-      </c>
-      <c r="F20" t="s">
+      <c r="I20" t="s">
         <v>113</v>
       </c>
-      <c r="G20" t="s">
-        <v>23</v>
-      </c>
-      <c r="H20" t="s">
-        <v>114</v>
-      </c>
-      <c r="I20" t="s">
-        <v>115</v>
-      </c>
       <c r="J20">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K20" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="L20" t="s">
-        <v>27</v>
+        <v>74</v>
       </c>
       <c r="M20" t="s">
         <v>28</v>
       </c>
       <c r="N20">
-        <v>2090</v>
+        <v>850</v>
       </c>
       <c r="O20">
-        <v>149</v>
+        <v>124</v>
       </c>
       <c r="P20">
         <v>6</v>
       </c>
       <c r="Q20">
+        <v>5100</v>
+      </c>
+      <c r="R20">
+        <v>744</v>
+      </c>
+      <c r="S20" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="21" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" t="s">
+        <v>114</v>
+      </c>
+      <c r="C21" t="s">
+        <v>54</v>
+      </c>
+      <c r="D21" t="s">
+        <v>115</v>
+      </c>
+      <c r="E21" t="s">
+        <v>67</v>
+      </c>
+      <c r="F21" t="s">
+        <v>78</v>
+      </c>
+      <c r="G21" t="s">
+        <v>23</v>
+      </c>
+      <c r="H21" t="s">
+        <v>79</v>
+      </c>
+      <c r="I21" t="s">
+        <v>80</v>
+      </c>
+      <c r="J21">
+        <v>3</v>
+      </c>
+      <c r="K21" t="s">
+        <v>41</v>
+      </c>
+      <c r="L21" t="s">
+        <v>27</v>
+      </c>
+      <c r="M21" t="s">
+        <v>28</v>
+      </c>
+      <c r="N21">
+        <v>2090</v>
+      </c>
+      <c r="O21">
+        <v>149</v>
+      </c>
+      <c r="P21">
+        <v>6</v>
+      </c>
+      <c r="Q21">
         <v>12540</v>
       </c>
-      <c r="R20">
+      <c r="R21">
         <v>894</v>
       </c>
-      <c r="S20" t="s">
-        <v>116</v>
+      <c r="S21" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(import): import full month August 2026 data (721 trips, 293 locations, 26 active quotations) from updated sheet
</commit_message>
<xml_diff>
--- a/august_import_files/MERCON_August_Quotations_Used_Only.xlsx
+++ b/august_import_files/MERCON_August_Quotations_Used_Only.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="347" uniqueCount="129">
   <si>
     <t>#</t>
   </si>
@@ -70,39 +70,45 @@
     <t>Status</t>
   </si>
   <si>
+    <t>91d5d96d-f96f-4651-adbd-f8456dc8fbcb</t>
+  </si>
+  <si>
+    <t>JDL</t>
+  </si>
+  <si>
+    <t>JDL | RIYADH SORTING CENTER -&gt; RIYADH STATION (SULAY/TUWAIQ/AZIZYAH/ALKHARJ) | 5M-5TON</t>
+  </si>
+  <si>
+    <t>RIYADH</t>
+  </si>
+  <si>
+    <t>—</t>
+  </si>
+  <si>
+    <t>5 TON</t>
+  </si>
+  <si>
+    <t>ROUND_TRIP</t>
+  </si>
+  <si>
+    <t>EXTRA</t>
+  </si>
+  <si>
+    <t>Active</t>
+  </si>
+  <si>
     <t>26044176-ecf4-45e6-8687-5d6b16aa4f41</t>
   </si>
   <si>
-    <t>JDL</t>
-  </si>
-  <si>
     <t>JDL | RIYADH SORTING CENTER -&gt; DUWADIMI | 5M-5TON</t>
   </si>
   <si>
-    <t>RIYADH</t>
-  </si>
-  <si>
-    <t>—</t>
-  </si>
-  <si>
     <t>DUWADIMI</t>
   </si>
   <si>
     <t>RIYADH → DUWADIMI</t>
   </si>
   <si>
-    <t>5 TON</t>
-  </si>
-  <si>
-    <t>ROUND_TRIP</t>
-  </si>
-  <si>
-    <t>EXTRA</t>
-  </si>
-  <si>
-    <t>Active</t>
-  </si>
-  <si>
     <t>e2e53349-db67-41d0-ab1a-cdd1a5b93753</t>
   </si>
   <si>
@@ -124,6 +130,42 @@
     <t>20 TON</t>
   </si>
   <si>
+    <t>ea082221-4a79-4a2e-b809-f442fee84c22</t>
+  </si>
+  <si>
+    <t>JDL | RIYADH -&gt; KHAMIS | 6.5M-10TON</t>
+  </si>
+  <si>
+    <t>KHAMIS</t>
+  </si>
+  <si>
+    <t>RIYADH → KHAMIS</t>
+  </si>
+  <si>
+    <t>10 TON</t>
+  </si>
+  <si>
+    <t>1d6cb12b-cd59-47d2-855c-b19cf7e377da</t>
+  </si>
+  <si>
+    <t>JDL | RIYADH -&gt; HAIL | 5M-5TON</t>
+  </si>
+  <si>
+    <t>BURAYDAH</t>
+  </si>
+  <si>
+    <t>HAIL</t>
+  </si>
+  <si>
+    <t>RIYADH → BURAYDAH → HAIL</t>
+  </si>
+  <si>
+    <t>c9f72037-f5cb-4a48-aa8a-4067b9a7623f</t>
+  </si>
+  <si>
+    <t>JDL | RIYADH -&gt; HAIL | 6.5M-10TON</t>
+  </si>
+  <si>
     <t>afc6e0d8-f2cd-45de-b1d3-2324ce572d06</t>
   </si>
   <si>
@@ -136,9 +178,6 @@
     <t>RIYADH → MADINA</t>
   </si>
   <si>
-    <t>10 TON</t>
-  </si>
-  <si>
     <t>043d05ac-4d17-4699-bff1-08cdf45e4869</t>
   </si>
   <si>
@@ -157,19 +196,22 @@
     <t>3-4 TON</t>
   </si>
   <si>
-    <t>18f96423-940c-4fa1-b18a-b6ccf379bc82</t>
-  </si>
-  <si>
-    <t>JDL | HAIL SORTING CENTER -&gt; QURAYYAT | 3TON/4TON</t>
-  </si>
-  <si>
-    <t>HAIL</t>
-  </si>
-  <si>
-    <t>QURAYYAT</t>
-  </si>
-  <si>
-    <t>HAIL → QURAYYAT</t>
+    <t>ecd70207-53a9-432a-86c0-32ce90d48d91</t>
+  </si>
+  <si>
+    <t>JDL | RIYADH SORTING CENTER -&gt; BURAYDAH | 5M-5TON</t>
+  </si>
+  <si>
+    <t>RIYADH → BURAYDAH</t>
+  </si>
+  <si>
+    <t>05627278-4ace-4504-923a-8c0951508e88</t>
+  </si>
+  <si>
+    <t>JDL | RIYADH -&gt; MAXIMUM 12H | 6.5M-10TON</t>
+  </si>
+  <si>
+    <t>SINGLE_TRIP</t>
   </si>
   <si>
     <t>38065f2c-3dd4-43d8-9ee3-4e203e62a42b</t>
@@ -193,19 +235,19 @@
     <t>iMile | INSIDE RIYADH -&gt; INSIDE RIYADH | 13.5M-20TON</t>
   </si>
   <si>
-    <t>e66e9210-f4a6-463b-80c6-a292aad63e55</t>
-  </si>
-  <si>
-    <t>iMile | KHAMIS MUSHAIT DISTIBUTION CENTRE -&gt; ABHA STATION | 6.5M-10TON</t>
+    <t>239d2a77-6e3d-42da-9bfc-db8dac32ed06</t>
+  </si>
+  <si>
+    <t>iMile | KHAMIS MUSHAIT DISTIBUTION CENTRE -&gt; JAZAN STATION | 13.5M-20TON</t>
   </si>
   <si>
     <t>KHAMIS MUSHAIT DISTIBUTION CENTRE</t>
   </si>
   <si>
-    <t>ABHA</t>
-  </si>
-  <si>
-    <t>KHAMIS MUSHAIT DISTIBUTION CENTRE → ABHA</t>
+    <t>JAZAN</t>
+  </si>
+  <si>
+    <t>KHAMIS MUSHAIT DISTIBUTION CENTRE → JAZAN</t>
   </si>
   <si>
     <t>f43d1d95-570c-477f-b5c5-682a6f974f82</t>
@@ -235,16 +277,109 @@
     <t>KHAMIS MUSHAIT DISTRIBUTION CENTRE → MUHAYIL</t>
   </si>
   <si>
-    <t>SINGLE_TRIP</t>
-  </si>
-  <si>
     <t>MONTHLY</t>
   </si>
   <si>
-    <t>61c3ba0d-9bbc-4198-aba9-ba57cc25d5af</t>
-  </si>
-  <si>
-    <t>iMile | RIYADH DISTRIBUTION CENTRE -&gt; AL BAHAH STATION | 6.5M-10TON</t>
+    <t>a51615b5-9ae7-4151-a854-a6972605499d</t>
+  </si>
+  <si>
+    <t>Shipa</t>
+  </si>
+  <si>
+    <t>Shipa | RIYADH -&gt; MAKKAH | 5 TON</t>
+  </si>
+  <si>
+    <t>RIYADH → MAKKAH</t>
+  </si>
+  <si>
+    <t>3ca8e844-de94-4f91-aa46-27d9b509e456</t>
+  </si>
+  <si>
+    <t>Shipa | RIYADH AIRPORT -&gt; RIYADH LOCAL | 10 TON</t>
+  </si>
+  <si>
+    <t>RIYADH AIRPORT</t>
+  </si>
+  <si>
+    <t>RIYADH LOCAL</t>
+  </si>
+  <si>
+    <t>RIYADH AIRPORT → RIYADH → RIYADH LOCAL</t>
+  </si>
+  <si>
+    <t>b5150f2f-cd3a-421b-b358-925943c90d19</t>
+  </si>
+  <si>
+    <t>Shipa | RIYADH -&gt; HAIL | 10 TON</t>
+  </si>
+  <si>
+    <t>RIYADH → HAIL</t>
+  </si>
+  <si>
+    <t>0e031238-7d8f-4aa7-8424-554aa546a212</t>
+  </si>
+  <si>
+    <t>Horizon</t>
+  </si>
+  <si>
+    <t>Horizon | RIYADH -&gt; DAMMAM ( KHOBAR ) | 10 TON</t>
+  </si>
+  <si>
+    <t>DAMMAM</t>
+  </si>
+  <si>
+    <t>RIYADH → DAMMAM</t>
+  </si>
+  <si>
+    <t>001742a5-1032-4108-b7d9-9a8670b7e1a2</t>
+  </si>
+  <si>
+    <t>Horizon | RIYADH -&gt; RIYADH LOCAL | 5 TON</t>
+  </si>
+  <si>
+    <t>RIYADH → RIYADH LOCAL</t>
+  </si>
+  <si>
+    <t>53e8f892-b5b2-499e-a4ff-737a528253d8</t>
+  </si>
+  <si>
+    <t>AKS</t>
+  </si>
+  <si>
+    <t>AKS | RIYADH -&gt; UNAIZA | LORRY</t>
+  </si>
+  <si>
+    <t>UNAIZA</t>
+  </si>
+  <si>
+    <t>RIYADH → UNAIZA</t>
+  </si>
+  <si>
+    <t>5eb9343b-23ae-4abf-b206-430a40ccdcc8</t>
+  </si>
+  <si>
+    <t>AKS | RIYADH -&gt; RIYADH LOCAL | LORRY</t>
+  </si>
+  <si>
+    <t>3e6af7f7-2ff4-4184-bcdc-706e10cd9899</t>
+  </si>
+  <si>
+    <t>AKS | RIYADH -&gt; RIYADH LOCAL | 40 FEET</t>
+  </si>
+  <si>
+    <t>40 FEET</t>
+  </si>
+  <si>
+    <t>f09a9847-8a4a-4c02-beb7-3b08ca81a182</t>
+  </si>
+  <si>
+    <t>AKS | RIYADH -&gt; DAMMAM | DYNA 3 TON</t>
+  </si>
+  <si>
+    <t>b1026a52-154d-4b50-a573-265c5e34f0d7</t>
+  </si>
+  <si>
+    <t>[HISTORICAL] iMile | RIYADH CENTRE -&gt; AL BAHAH STATION | 6.5M-10TON</t>
   </si>
   <si>
     <t>AL</t>
@@ -256,116 +391,20 @@
     <t>RIYADH CENTRE → AL → AL BAHAH STATION</t>
   </si>
   <si>
-    <t>a51615b5-9ae7-4151-a854-a6972605499d</t>
-  </si>
-  <si>
-    <t>Shipa</t>
-  </si>
-  <si>
-    <t>Shipa | RIYADH -&gt; MAKKAH | 5 TON</t>
-  </si>
-  <si>
-    <t>RIYADH → MAKKAH</t>
-  </si>
-  <si>
-    <t>3ca8e844-de94-4f91-aa46-27d9b509e456</t>
-  </si>
-  <si>
-    <t>Shipa | RIYADH AIRPORT -&gt; RIYADH LOCAL | 10 TON</t>
-  </si>
-  <si>
-    <t>RIYADH AIRPORT</t>
-  </si>
-  <si>
-    <t>RIYADH LOCAL</t>
-  </si>
-  <si>
-    <t>RIYADH AIRPORT → RIYADH → RIYADH LOCAL</t>
-  </si>
-  <si>
-    <t>134d2b85-2858-4b4e-ab08-01128bfd52f9</t>
-  </si>
-  <si>
-    <t>Shipa | RIYADH -&gt; TAIF-MAKKAH | 5 TON</t>
-  </si>
-  <si>
-    <t>TAIF</t>
-  </si>
-  <si>
-    <t>RIYADH → TAIF → MAKKAH</t>
-  </si>
-  <si>
-    <t>869ee64a-82fd-4ef3-b224-0fe6b86ecfb9</t>
-  </si>
-  <si>
-    <t>Shipa | RUH -&gt; JED | 5 TON</t>
-  </si>
-  <si>
-    <t>RUH</t>
-  </si>
-  <si>
-    <t>JED</t>
-  </si>
-  <si>
-    <t>RUH → JED</t>
-  </si>
-  <si>
-    <t>53e8f892-b5b2-499e-a4ff-737a528253d8</t>
-  </si>
-  <si>
-    <t>AKS</t>
-  </si>
-  <si>
-    <t>AKS | RIYADH -&gt; UNAIZA | LORRY</t>
-  </si>
-  <si>
-    <t>UNAIZA</t>
-  </si>
-  <si>
-    <t>RIYADH → UNAIZA</t>
-  </si>
-  <si>
-    <t>5eb9343b-23ae-4abf-b206-430a40ccdcc8</t>
-  </si>
-  <si>
-    <t>AKS | RIYADH -&gt; RIYADH LOCAL | LORRY</t>
-  </si>
-  <si>
-    <t>RIYADH → RIYADH LOCAL</t>
-  </si>
-  <si>
-    <t>3e6af7f7-2ff4-4184-bcdc-706e10cd9899</t>
-  </si>
-  <si>
-    <t>AKS | RIYADH -&gt; RIYADH LOCAL | 40 FEET</t>
-  </si>
-  <si>
-    <t>40 FEET</t>
-  </si>
-  <si>
-    <t>f09a9847-8a4a-4c02-beb7-3b08ca81a182</t>
-  </si>
-  <si>
-    <t>AKS | RIYADH -&gt; DAMMAM | DYNA 3 TON</t>
-  </si>
-  <si>
-    <t>DAMMAM</t>
-  </si>
-  <si>
-    <t>RIYADH → DAMMAM</t>
-  </si>
-  <si>
-    <t>b1026a52-154d-4b50-a573-265c5e34f0d7</t>
-  </si>
-  <si>
-    <t>[HISTORICAL] iMile | RIYADH CENTRE -&gt; AL BAHAH STATION | 6.5M-10TON</t>
+    <t>10d9ff1f-07de-4fa8-acf4-bbd8d2592110</t>
+  </si>
+  <si>
+    <t>Illegal Cross Customer Quote</t>
+  </si>
+  <si>
+    <t/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -373,23 +412,13 @@
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
-    <font>
-      <b/>
-      <color rgb="FFFFFF"/>
-      <sz val="11"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="3E3C3D"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -404,11 +433,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -748,85 +774,65 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:S21"/>
+  <dimension ref="A1:S27"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
-  <cols>
-    <col min="1" max="1" width="16" customWidth="1"/>
-    <col min="2" max="2" width="40" customWidth="1"/>
-    <col min="3" max="3" width="17" customWidth="1"/>
-    <col min="4" max="4" width="50" customWidth="1"/>
-    <col min="5" max="5" width="38" customWidth="1"/>
-    <col min="6" max="6" width="17" customWidth="1"/>
-    <col min="7" max="8" width="23" customWidth="1"/>
-    <col min="9" max="9" width="50" customWidth="1"/>
-    <col min="10" max="10" width="16" customWidth="1"/>
-    <col min="11" max="11" width="17" customWidth="1"/>
-    <col min="12" max="12" width="16" customWidth="1"/>
-    <col min="13" max="13" width="18" customWidth="1"/>
-    <col min="14" max="14" width="22" customWidth="1"/>
-    <col min="15" max="15" width="23" customWidth="1"/>
-    <col min="16" max="16" width="25" customWidth="1"/>
-    <col min="17" max="17" width="30" customWidth="1"/>
-    <col min="18" max="18" width="34" customWidth="1"/>
-    <col min="19" max="19" width="16" customWidth="1"/>
-  </cols>
   <sheetData>
-    <row r="1" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
     </row>
@@ -853,40 +859,40 @@
         <v>23</v>
       </c>
       <c r="H2" t="s">
+        <v>23</v>
+      </c>
+      <c r="I2" t="s">
+        <v>22</v>
+      </c>
+      <c r="J2">
+        <v>1</v>
+      </c>
+      <c r="K2" t="s">
         <v>24</v>
       </c>
-      <c r="I2" t="s">
+      <c r="L2" t="s">
         <v>25</v>
       </c>
-      <c r="J2">
-        <v>2</v>
-      </c>
-      <c r="K2" t="s">
-        <v>26</v>
-      </c>
-      <c r="L2" t="s">
-        <v>27</v>
-      </c>
       <c r="M2" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="N2">
-        <v>695</v>
-      </c>
-      <c r="O2">
-        <v>55</v>
+        <v>320</v>
+      </c>
+      <c r="O2" t="s">
+        <v>23</v>
       </c>
       <c r="P2">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="Q2">
-        <v>15290</v>
-      </c>
-      <c r="R2">
-        <v>1210</v>
+        <v>320</v>
+      </c>
+      <c r="R2" t="s">
+        <v>23</v>
       </c>
       <c r="S2" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.25">
@@ -894,58 +900,58 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C3" t="s">
         <v>20</v>
       </c>
       <c r="D3" t="s">
+        <v>29</v>
+      </c>
+      <c r="E3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H3" t="s">
+        <v>30</v>
+      </c>
+      <c r="I3" t="s">
         <v>31</v>
       </c>
-      <c r="E3" t="s">
-        <v>32</v>
-      </c>
-      <c r="F3" t="s">
-        <v>33</v>
-      </c>
-      <c r="G3" t="s">
-        <v>34</v>
-      </c>
-      <c r="H3" t="s">
-        <v>34</v>
-      </c>
-      <c r="I3" t="s">
-        <v>35</v>
-      </c>
       <c r="J3">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K3" t="s">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="L3" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="M3" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="N3">
-        <v>1150</v>
+        <v>695</v>
       </c>
       <c r="O3">
-        <v>64</v>
+        <v>55</v>
       </c>
       <c r="P3">
-        <v>4</v>
+        <v>31</v>
       </c>
       <c r="Q3">
-        <v>4600</v>
+        <v>21545</v>
       </c>
       <c r="R3">
-        <v>256</v>
+        <v>1705</v>
       </c>
       <c r="S3" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.25">
@@ -953,58 +959,58 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="C4" t="s">
         <v>20</v>
       </c>
       <c r="D4" t="s">
+        <v>33</v>
+      </c>
+      <c r="E4" t="s">
+        <v>34</v>
+      </c>
+      <c r="F4" t="s">
+        <v>35</v>
+      </c>
+      <c r="G4" t="s">
+        <v>36</v>
+      </c>
+      <c r="H4" t="s">
+        <v>36</v>
+      </c>
+      <c r="I4" t="s">
+        <v>37</v>
+      </c>
+      <c r="J4">
+        <v>4</v>
+      </c>
+      <c r="K4" t="s">
         <v>38</v>
       </c>
-      <c r="E4" t="s">
-        <v>22</v>
-      </c>
-      <c r="F4" t="s">
-        <v>23</v>
-      </c>
-      <c r="G4" t="s">
-        <v>23</v>
-      </c>
-      <c r="H4" t="s">
-        <v>39</v>
-      </c>
-      <c r="I4" t="s">
-        <v>40</v>
-      </c>
-      <c r="J4">
-        <v>2</v>
-      </c>
-      <c r="K4" t="s">
-        <v>41</v>
-      </c>
       <c r="L4" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="M4" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="N4">
-        <v>1665</v>
+        <v>1150</v>
       </c>
       <c r="O4">
-        <v>144</v>
+        <v>64</v>
       </c>
       <c r="P4">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Q4">
-        <v>6660</v>
+        <v>3450</v>
       </c>
       <c r="R4">
-        <v>576</v>
+        <v>192</v>
       </c>
       <c r="S4" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
@@ -1012,16 +1018,16 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="C5" t="s">
         <v>20</v>
       </c>
       <c r="D5" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="E5" t="s">
-        <v>44</v>
+        <v>22</v>
       </c>
       <c r="F5" t="s">
         <v>23</v>
@@ -1030,40 +1036,40 @@
         <v>23</v>
       </c>
       <c r="H5" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="I5" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="J5">
         <v>2</v>
       </c>
       <c r="K5" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="L5" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="M5" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="N5">
-        <v>530</v>
-      </c>
-      <c r="O5">
-        <v>50</v>
+        <v>1800</v>
+      </c>
+      <c r="O5" t="s">
+        <v>23</v>
       </c>
       <c r="P5">
-        <v>22</v>
+        <v>2</v>
       </c>
       <c r="Q5">
-        <v>11660</v>
-      </c>
-      <c r="R5">
-        <v>1100</v>
+        <v>3600</v>
+      </c>
+      <c r="R5" t="s">
+        <v>23</v>
       </c>
       <c r="S5" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.25">
@@ -1071,58 +1077,58 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="C6" t="s">
         <v>20</v>
       </c>
       <c r="D6" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="E6" t="s">
-        <v>50</v>
+        <v>22</v>
       </c>
       <c r="F6" t="s">
-        <v>23</v>
+        <v>46</v>
       </c>
       <c r="G6" t="s">
         <v>23</v>
       </c>
       <c r="H6" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="I6" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="J6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K6" t="s">
-        <v>47</v>
+        <v>24</v>
       </c>
       <c r="L6" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="M6" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="N6">
-        <v>1240</v>
+        <v>1200</v>
       </c>
       <c r="O6">
         <v>105</v>
       </c>
       <c r="P6">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="Q6">
-        <v>27280</v>
+        <v>1200</v>
       </c>
       <c r="R6">
-        <v>2310</v>
+        <v>105</v>
       </c>
       <c r="S6" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.25">
@@ -1130,58 +1136,58 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="C7" t="s">
-        <v>54</v>
+        <v>20</v>
       </c>
       <c r="D7" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="E7" t="s">
-        <v>56</v>
+        <v>22</v>
       </c>
       <c r="F7" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
       <c r="G7" t="s">
         <v>23</v>
       </c>
       <c r="H7" t="s">
-        <v>22</v>
+        <v>47</v>
       </c>
       <c r="I7" t="s">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="J7">
         <v>3</v>
       </c>
       <c r="K7" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="L7" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="M7" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="N7">
-        <v>545</v>
+        <v>1400</v>
       </c>
       <c r="O7">
-        <v>60</v>
+        <v>105</v>
       </c>
       <c r="P7">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="Q7">
-        <v>5450</v>
+        <v>16800</v>
       </c>
       <c r="R7">
-        <v>600</v>
+        <v>1260</v>
       </c>
       <c r="S7" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.25">
@@ -1189,58 +1195,58 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="C8" t="s">
+        <v>20</v>
+      </c>
+      <c r="D8" t="s">
+        <v>52</v>
+      </c>
+      <c r="E8" t="s">
+        <v>22</v>
+      </c>
+      <c r="F8" t="s">
+        <v>23</v>
+      </c>
+      <c r="G8" t="s">
+        <v>23</v>
+      </c>
+      <c r="H8" t="s">
+        <v>53</v>
+      </c>
+      <c r="I8" t="s">
         <v>54</v>
       </c>
-      <c r="D8" t="s">
-        <v>59</v>
-      </c>
-      <c r="E8" t="s">
-        <v>56</v>
-      </c>
-      <c r="F8" t="s">
-        <v>56</v>
-      </c>
-      <c r="G8" t="s">
-        <v>23</v>
-      </c>
-      <c r="H8" t="s">
-        <v>22</v>
-      </c>
-      <c r="I8" t="s">
-        <v>57</v>
-      </c>
       <c r="J8">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K8" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="L8" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="M8" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="N8">
-        <v>1050</v>
+        <v>1665</v>
       </c>
       <c r="O8">
-        <v>64</v>
+        <v>144</v>
       </c>
       <c r="P8">
         <v>2</v>
       </c>
       <c r="Q8">
-        <v>2100</v>
+        <v>3330</v>
       </c>
       <c r="R8">
-        <v>128</v>
+        <v>288</v>
       </c>
       <c r="S8" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.25">
@@ -1248,16 +1254,16 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="C9" t="s">
-        <v>54</v>
+        <v>20</v>
       </c>
       <c r="D9" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="E9" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="F9" t="s">
         <v>23</v>
@@ -1266,40 +1272,40 @@
         <v>23</v>
       </c>
       <c r="H9" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="I9" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="J9">
         <v>2</v>
       </c>
       <c r="K9" t="s">
-        <v>41</v>
+        <v>60</v>
       </c>
       <c r="L9" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="M9" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="N9">
-        <v>624</v>
+        <v>530</v>
       </c>
       <c r="O9">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="P9">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="Q9">
-        <v>13728</v>
+        <v>16430</v>
       </c>
       <c r="R9">
-        <v>1320</v>
+        <v>1550</v>
       </c>
       <c r="S9" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.25">
@@ -1307,16 +1313,16 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="C10" t="s">
-        <v>54</v>
+        <v>20</v>
       </c>
       <c r="D10" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="E10" t="s">
-        <v>67</v>
+        <v>22</v>
       </c>
       <c r="F10" t="s">
         <v>23</v>
@@ -1325,40 +1331,40 @@
         <v>23</v>
       </c>
       <c r="H10" t="s">
-        <v>24</v>
+        <v>46</v>
       </c>
       <c r="I10" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="J10">
         <v>2</v>
       </c>
       <c r="K10" t="s">
-        <v>41</v>
+        <v>24</v>
       </c>
       <c r="L10" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="M10" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="N10">
-        <v>1015</v>
-      </c>
-      <c r="O10">
-        <v>64</v>
+        <v>710</v>
+      </c>
+      <c r="O10" t="s">
+        <v>23</v>
       </c>
       <c r="P10">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="Q10">
-        <v>4060</v>
-      </c>
-      <c r="R10">
-        <v>256</v>
+        <v>710</v>
+      </c>
+      <c r="R10" t="s">
+        <v>23</v>
       </c>
       <c r="S10" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.25">
@@ -1366,16 +1372,16 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="C11" t="s">
-        <v>54</v>
+        <v>20</v>
       </c>
       <c r="D11" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="E11" t="s">
-        <v>71</v>
+        <v>22</v>
       </c>
       <c r="F11" t="s">
         <v>23</v>
@@ -1384,40 +1390,40 @@
         <v>23</v>
       </c>
       <c r="H11" t="s">
-        <v>72</v>
+        <v>23</v>
       </c>
       <c r="I11" t="s">
-        <v>73</v>
+        <v>22</v>
       </c>
       <c r="J11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K11" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="L11" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
       <c r="M11" t="s">
-        <v>75</v>
+        <v>26</v>
       </c>
       <c r="N11">
-        <v>499</v>
-      </c>
-      <c r="O11">
-        <v>50</v>
+        <v>550</v>
+      </c>
+      <c r="O11" t="s">
+        <v>23</v>
       </c>
       <c r="P11">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="Q11">
-        <v>10978</v>
-      </c>
-      <c r="R11">
-        <v>1100</v>
+        <v>550</v>
+      </c>
+      <c r="R11" t="s">
+        <v>23</v>
       </c>
       <c r="S11" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="12" spans="1:19" x14ac:dyDescent="0.25">
@@ -1425,58 +1431,58 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>76</v>
+        <v>67</v>
       </c>
       <c r="C12" t="s">
-        <v>54</v>
+        <v>68</v>
       </c>
       <c r="D12" t="s">
-        <v>77</v>
+        <v>69</v>
       </c>
       <c r="E12" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="F12" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="G12" t="s">
         <v>23</v>
       </c>
       <c r="H12" t="s">
-        <v>79</v>
+        <v>22</v>
       </c>
       <c r="I12" t="s">
-        <v>80</v>
+        <v>71</v>
       </c>
       <c r="J12">
         <v>3</v>
       </c>
       <c r="K12" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="L12" t="s">
-        <v>74</v>
+        <v>25</v>
       </c>
       <c r="M12" t="s">
-        <v>75</v>
+        <v>26</v>
       </c>
       <c r="N12">
-        <v>1750</v>
+        <v>545</v>
       </c>
       <c r="O12">
-        <v>149</v>
+        <v>60</v>
       </c>
       <c r="P12">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="Q12">
-        <v>38500</v>
+        <v>4360</v>
       </c>
       <c r="R12">
-        <v>3278</v>
+        <v>480</v>
       </c>
       <c r="S12" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="13" spans="1:19" x14ac:dyDescent="0.25">
@@ -1484,58 +1490,58 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>81</v>
+        <v>72</v>
       </c>
       <c r="C13" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="D13" t="s">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="E13" t="s">
+        <v>70</v>
+      </c>
+      <c r="F13" t="s">
+        <v>70</v>
+      </c>
+      <c r="G13" t="s">
+        <v>23</v>
+      </c>
+      <c r="H13" t="s">
         <v>22</v>
       </c>
-      <c r="F13" t="s">
-        <v>23</v>
-      </c>
-      <c r="G13" t="s">
-        <v>23</v>
-      </c>
-      <c r="H13" t="s">
-        <v>45</v>
-      </c>
       <c r="I13" t="s">
-        <v>84</v>
+        <v>71</v>
       </c>
       <c r="J13">
+        <v>3</v>
+      </c>
+      <c r="K13" t="s">
+        <v>38</v>
+      </c>
+      <c r="L13" t="s">
+        <v>25</v>
+      </c>
+      <c r="M13" t="s">
+        <v>26</v>
+      </c>
+      <c r="N13">
+        <v>1050</v>
+      </c>
+      <c r="O13">
+        <v>64</v>
+      </c>
+      <c r="P13">
         <v>2</v>
       </c>
-      <c r="K13" t="s">
-        <v>26</v>
-      </c>
-      <c r="L13" t="s">
-        <v>74</v>
-      </c>
-      <c r="M13" t="s">
-        <v>28</v>
-      </c>
-      <c r="N13">
-        <v>1375</v>
-      </c>
-      <c r="O13">
-        <v>1200</v>
-      </c>
-      <c r="P13">
-        <v>4</v>
-      </c>
       <c r="Q13">
-        <v>5500</v>
+        <v>2100</v>
       </c>
       <c r="R13">
-        <v>4800</v>
+        <v>128</v>
       </c>
       <c r="S13" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="14" spans="1:19" x14ac:dyDescent="0.25">
@@ -1543,58 +1549,58 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>85</v>
+        <v>74</v>
       </c>
       <c r="C14" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="D14" t="s">
-        <v>86</v>
+        <v>75</v>
       </c>
       <c r="E14" t="s">
-        <v>87</v>
+        <v>76</v>
       </c>
       <c r="F14" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G14" t="s">
         <v>23</v>
       </c>
       <c r="H14" t="s">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="I14" t="s">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="J14">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K14" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="L14" t="s">
-        <v>74</v>
+        <v>25</v>
       </c>
       <c r="M14" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="N14">
-        <v>500</v>
+        <v>1750</v>
       </c>
       <c r="O14">
-        <v>45</v>
+        <v>149</v>
       </c>
       <c r="P14">
-        <v>4</v>
+        <v>31</v>
       </c>
       <c r="Q14">
-        <v>2000</v>
+        <v>54250</v>
       </c>
       <c r="R14">
-        <v>180</v>
+        <v>4619</v>
       </c>
       <c r="S14" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="15" spans="1:19" x14ac:dyDescent="0.25">
@@ -1602,58 +1608,58 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="C15" t="s">
+        <v>68</v>
+      </c>
+      <c r="D15" t="s">
+        <v>80</v>
+      </c>
+      <c r="E15" t="s">
+        <v>81</v>
+      </c>
+      <c r="F15" t="s">
+        <v>23</v>
+      </c>
+      <c r="G15" t="s">
+        <v>23</v>
+      </c>
+      <c r="H15" t="s">
+        <v>30</v>
+      </c>
+      <c r="I15" t="s">
         <v>82</v>
       </c>
-      <c r="D15" t="s">
-        <v>91</v>
-      </c>
-      <c r="E15" t="s">
-        <v>22</v>
-      </c>
-      <c r="F15" t="s">
-        <v>92</v>
-      </c>
-      <c r="G15" t="s">
-        <v>23</v>
-      </c>
-      <c r="H15" t="s">
-        <v>45</v>
-      </c>
-      <c r="I15" t="s">
-        <v>93</v>
-      </c>
       <c r="J15">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K15" t="s">
-        <v>26</v>
+        <v>43</v>
       </c>
       <c r="L15" t="s">
-        <v>74</v>
+        <v>25</v>
       </c>
       <c r="M15" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="N15">
-        <v>1500</v>
+        <v>1015</v>
       </c>
       <c r="O15">
-        <v>149</v>
+        <v>64</v>
       </c>
       <c r="P15">
-        <v>22</v>
+        <v>2</v>
       </c>
       <c r="Q15">
-        <v>33000</v>
+        <v>2030</v>
       </c>
       <c r="R15">
-        <v>3278</v>
+        <v>128</v>
       </c>
       <c r="S15" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.25">
@@ -1661,16 +1667,16 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>94</v>
+        <v>83</v>
       </c>
       <c r="C16" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="D16" t="s">
-        <v>95</v>
+        <v>84</v>
       </c>
       <c r="E16" t="s">
-        <v>96</v>
+        <v>85</v>
       </c>
       <c r="F16" t="s">
         <v>23</v>
@@ -1679,40 +1685,40 @@
         <v>23</v>
       </c>
       <c r="H16" t="s">
-        <v>97</v>
+        <v>86</v>
       </c>
       <c r="I16" t="s">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="J16">
         <v>2</v>
       </c>
       <c r="K16" t="s">
-        <v>26</v>
+        <v>43</v>
       </c>
       <c r="L16" t="s">
-        <v>27</v>
+        <v>66</v>
       </c>
       <c r="M16" t="s">
-        <v>75</v>
+        <v>88</v>
       </c>
       <c r="N16">
-        <v>49850</v>
+        <v>499</v>
       </c>
       <c r="O16">
-        <v>149</v>
+        <v>50</v>
       </c>
       <c r="P16">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="Q16">
-        <v>2193400</v>
+        <v>15469</v>
       </c>
       <c r="R16">
-        <v>6556</v>
+        <v>1550</v>
       </c>
       <c r="S16" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.25">
@@ -1720,13 +1726,13 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="C17" t="s">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="D17" t="s">
-        <v>101</v>
+        <v>91</v>
       </c>
       <c r="E17" t="s">
         <v>22</v>
@@ -1738,40 +1744,40 @@
         <v>23</v>
       </c>
       <c r="H17" t="s">
-        <v>102</v>
+        <v>58</v>
       </c>
       <c r="I17" t="s">
-        <v>103</v>
+        <v>92</v>
       </c>
       <c r="J17">
         <v>2</v>
       </c>
       <c r="K17" t="s">
-        <v>41</v>
+        <v>24</v>
       </c>
       <c r="L17" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
       <c r="M17" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="N17">
-        <v>1300</v>
+        <v>1375</v>
       </c>
       <c r="O17">
-        <v>1650</v>
+        <v>1200</v>
       </c>
       <c r="P17">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q17">
-        <v>2600</v>
+        <v>4125</v>
       </c>
       <c r="R17">
-        <v>3300</v>
+        <v>3600</v>
       </c>
       <c r="S17" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="18" spans="1:19" x14ac:dyDescent="0.25">
@@ -1779,58 +1785,58 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>104</v>
+        <v>93</v>
       </c>
       <c r="C18" t="s">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="D18" t="s">
-        <v>105</v>
+        <v>94</v>
       </c>
       <c r="E18" t="s">
+        <v>95</v>
+      </c>
+      <c r="F18" t="s">
         <v>22</v>
       </c>
-      <c r="F18" t="s">
-        <v>23</v>
-      </c>
       <c r="G18" t="s">
         <v>23</v>
       </c>
       <c r="H18" t="s">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="I18" t="s">
-        <v>106</v>
+        <v>97</v>
       </c>
       <c r="J18">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K18" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="L18" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
       <c r="M18" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="N18">
-        <v>450</v>
+        <v>500</v>
       </c>
       <c r="O18">
-        <v>185</v>
+        <v>45</v>
       </c>
       <c r="P18">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q18">
-        <v>900</v>
+        <v>1500</v>
       </c>
       <c r="R18">
-        <v>370</v>
+        <v>135</v>
       </c>
       <c r="S18" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="19" spans="1:19" x14ac:dyDescent="0.25">
@@ -1838,13 +1844,13 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>107</v>
+        <v>98</v>
       </c>
       <c r="C19" t="s">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="D19" t="s">
-        <v>108</v>
+        <v>99</v>
       </c>
       <c r="E19" t="s">
         <v>22</v>
@@ -1856,40 +1862,40 @@
         <v>23</v>
       </c>
       <c r="H19" t="s">
-        <v>88</v>
+        <v>47</v>
       </c>
       <c r="I19" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="J19">
         <v>2</v>
       </c>
       <c r="K19" t="s">
-        <v>109</v>
+        <v>43</v>
       </c>
       <c r="L19" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
       <c r="M19" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="N19">
-        <v>900</v>
-      </c>
-      <c r="O19">
-        <v>1250</v>
+        <v>1550</v>
+      </c>
+      <c r="O19" t="s">
+        <v>23</v>
       </c>
       <c r="P19">
-        <v>4</v>
+        <v>29</v>
       </c>
       <c r="Q19">
-        <v>3600</v>
-      </c>
-      <c r="R19">
-        <v>5000</v>
+        <v>44950</v>
+      </c>
+      <c r="R19" t="s">
+        <v>23</v>
       </c>
       <c r="S19" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="20" spans="1:19" x14ac:dyDescent="0.25">
@@ -1897,13 +1903,13 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>110</v>
+        <v>101</v>
       </c>
       <c r="C20" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D20" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="E20" t="s">
         <v>22</v>
@@ -1915,40 +1921,40 @@
         <v>23</v>
       </c>
       <c r="H20" t="s">
-        <v>112</v>
+        <v>104</v>
       </c>
       <c r="I20" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="J20">
         <v>2</v>
       </c>
       <c r="K20" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="L20" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
       <c r="M20" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="N20">
-        <v>850</v>
-      </c>
-      <c r="O20">
-        <v>124</v>
+        <v>1345</v>
+      </c>
+      <c r="O20" t="s">
+        <v>23</v>
       </c>
       <c r="P20">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="Q20">
-        <v>5100</v>
-      </c>
-      <c r="R20">
-        <v>744</v>
+        <v>1345</v>
+      </c>
+      <c r="R20" t="s">
+        <v>23</v>
       </c>
       <c r="S20" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="21" spans="1:19" x14ac:dyDescent="0.25">
@@ -1956,58 +1962,412 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
+        <v>106</v>
+      </c>
+      <c r="C21" t="s">
+        <v>102</v>
+      </c>
+      <c r="D21" t="s">
+        <v>107</v>
+      </c>
+      <c r="E21" t="s">
+        <v>22</v>
+      </c>
+      <c r="F21" t="s">
+        <v>23</v>
+      </c>
+      <c r="G21" t="s">
+        <v>23</v>
+      </c>
+      <c r="H21" t="s">
+        <v>96</v>
+      </c>
+      <c r="I21" t="s">
+        <v>108</v>
+      </c>
+      <c r="J21">
+        <v>2</v>
+      </c>
+      <c r="K21" t="s">
+        <v>24</v>
+      </c>
+      <c r="L21" t="s">
+        <v>66</v>
+      </c>
+      <c r="M21" t="s">
+        <v>26</v>
+      </c>
+      <c r="N21">
+        <v>350</v>
+      </c>
+      <c r="O21" t="s">
+        <v>23</v>
+      </c>
+      <c r="P21">
+        <v>5</v>
+      </c>
+      <c r="Q21">
+        <v>1750</v>
+      </c>
+      <c r="R21" t="s">
+        <v>23</v>
+      </c>
+      <c r="S21" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="22" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" t="s">
+        <v>109</v>
+      </c>
+      <c r="C22" t="s">
+        <v>110</v>
+      </c>
+      <c r="D22" t="s">
+        <v>111</v>
+      </c>
+      <c r="E22" t="s">
+        <v>22</v>
+      </c>
+      <c r="F22" t="s">
+        <v>23</v>
+      </c>
+      <c r="G22" t="s">
+        <v>23</v>
+      </c>
+      <c r="H22" t="s">
+        <v>112</v>
+      </c>
+      <c r="I22" t="s">
+        <v>113</v>
+      </c>
+      <c r="J22">
+        <v>2</v>
+      </c>
+      <c r="K22" t="s">
+        <v>43</v>
+      </c>
+      <c r="L22" t="s">
+        <v>66</v>
+      </c>
+      <c r="M22" t="s">
+        <v>26</v>
+      </c>
+      <c r="N22">
+        <v>1300</v>
+      </c>
+      <c r="O22">
+        <v>1650</v>
+      </c>
+      <c r="P22">
+        <v>1</v>
+      </c>
+      <c r="Q22">
+        <v>1300</v>
+      </c>
+      <c r="R22">
+        <v>1650</v>
+      </c>
+      <c r="S22" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="23" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" t="s">
         <v>114</v>
       </c>
-      <c r="C21" t="s">
-        <v>54</v>
-      </c>
-      <c r="D21" t="s">
+      <c r="C23" t="s">
+        <v>110</v>
+      </c>
+      <c r="D23" t="s">
         <v>115</v>
       </c>
-      <c r="E21" t="s">
-        <v>67</v>
-      </c>
-      <c r="F21" t="s">
-        <v>78</v>
-      </c>
-      <c r="G21" t="s">
-        <v>23</v>
-      </c>
-      <c r="H21" t="s">
-        <v>79</v>
-      </c>
-      <c r="I21" t="s">
-        <v>80</v>
-      </c>
-      <c r="J21">
+      <c r="E23" t="s">
+        <v>22</v>
+      </c>
+      <c r="F23" t="s">
+        <v>23</v>
+      </c>
+      <c r="G23" t="s">
+        <v>23</v>
+      </c>
+      <c r="H23" t="s">
+        <v>96</v>
+      </c>
+      <c r="I23" t="s">
+        <v>108</v>
+      </c>
+      <c r="J23">
+        <v>2</v>
+      </c>
+      <c r="K23" t="s">
+        <v>43</v>
+      </c>
+      <c r="L23" t="s">
+        <v>66</v>
+      </c>
+      <c r="M23" t="s">
+        <v>26</v>
+      </c>
+      <c r="N23">
+        <v>450</v>
+      </c>
+      <c r="O23">
+        <v>185</v>
+      </c>
+      <c r="P23">
+        <v>2</v>
+      </c>
+      <c r="Q23">
+        <v>900</v>
+      </c>
+      <c r="R23">
+        <v>370</v>
+      </c>
+      <c r="S23" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="24" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" t="s">
+        <v>116</v>
+      </c>
+      <c r="C24" t="s">
+        <v>110</v>
+      </c>
+      <c r="D24" t="s">
+        <v>117</v>
+      </c>
+      <c r="E24" t="s">
+        <v>22</v>
+      </c>
+      <c r="F24" t="s">
+        <v>23</v>
+      </c>
+      <c r="G24" t="s">
+        <v>23</v>
+      </c>
+      <c r="H24" t="s">
+        <v>96</v>
+      </c>
+      <c r="I24" t="s">
+        <v>108</v>
+      </c>
+      <c r="J24">
+        <v>2</v>
+      </c>
+      <c r="K24" t="s">
+        <v>118</v>
+      </c>
+      <c r="L24" t="s">
+        <v>66</v>
+      </c>
+      <c r="M24" t="s">
+        <v>26</v>
+      </c>
+      <c r="N24">
+        <v>900</v>
+      </c>
+      <c r="O24">
+        <v>1250</v>
+      </c>
+      <c r="P24">
+        <v>5</v>
+      </c>
+      <c r="Q24">
+        <v>4500</v>
+      </c>
+      <c r="R24">
+        <v>6250</v>
+      </c>
+      <c r="S24" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="25" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" t="s">
+        <v>119</v>
+      </c>
+      <c r="C25" t="s">
+        <v>110</v>
+      </c>
+      <c r="D25" t="s">
+        <v>120</v>
+      </c>
+      <c r="E25" t="s">
+        <v>22</v>
+      </c>
+      <c r="F25" t="s">
+        <v>23</v>
+      </c>
+      <c r="G25" t="s">
+        <v>23</v>
+      </c>
+      <c r="H25" t="s">
+        <v>104</v>
+      </c>
+      <c r="I25" t="s">
+        <v>105</v>
+      </c>
+      <c r="J25">
+        <v>2</v>
+      </c>
+      <c r="K25" t="s">
+        <v>60</v>
+      </c>
+      <c r="L25" t="s">
+        <v>66</v>
+      </c>
+      <c r="M25" t="s">
+        <v>26</v>
+      </c>
+      <c r="N25">
+        <v>850</v>
+      </c>
+      <c r="O25">
+        <v>124</v>
+      </c>
+      <c r="P25">
+        <v>6</v>
+      </c>
+      <c r="Q25">
+        <v>5100</v>
+      </c>
+      <c r="R25">
+        <v>744</v>
+      </c>
+      <c r="S25" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="26" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26" t="s">
+        <v>121</v>
+      </c>
+      <c r="C26" t="s">
+        <v>68</v>
+      </c>
+      <c r="D26" t="s">
+        <v>122</v>
+      </c>
+      <c r="E26" t="s">
+        <v>81</v>
+      </c>
+      <c r="F26" t="s">
+        <v>123</v>
+      </c>
+      <c r="G26" t="s">
+        <v>23</v>
+      </c>
+      <c r="H26" t="s">
+        <v>124</v>
+      </c>
+      <c r="I26" t="s">
+        <v>125</v>
+      </c>
+      <c r="J26">
         <v>3</v>
       </c>
-      <c r="K21" t="s">
-        <v>41</v>
-      </c>
-      <c r="L21" t="s">
-        <v>27</v>
-      </c>
-      <c r="M21" t="s">
-        <v>28</v>
-      </c>
-      <c r="N21">
+      <c r="K26" t="s">
+        <v>43</v>
+      </c>
+      <c r="L26" t="s">
+        <v>25</v>
+      </c>
+      <c r="M26" t="s">
+        <v>26</v>
+      </c>
+      <c r="N26">
         <v>2090</v>
       </c>
-      <c r="O21">
+      <c r="O26">
         <v>149</v>
       </c>
-      <c r="P21">
-        <v>6</v>
-      </c>
-      <c r="Q21">
-        <v>12540</v>
-      </c>
-      <c r="R21">
-        <v>894</v>
-      </c>
-      <c r="S21" t="s">
-        <v>29</v>
+      <c r="P26">
+        <v>5</v>
+      </c>
+      <c r="Q26">
+        <v>10450</v>
+      </c>
+      <c r="R26">
+        <v>745</v>
+      </c>
+      <c r="S26" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="27" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27" t="s">
+        <v>126</v>
+      </c>
+      <c r="C27" t="s">
+        <v>20</v>
+      </c>
+      <c r="D27" t="s">
+        <v>127</v>
+      </c>
+      <c r="E27" t="s">
+        <v>23</v>
+      </c>
+      <c r="F27" t="s">
+        <v>23</v>
+      </c>
+      <c r="G27" t="s">
+        <v>23</v>
+      </c>
+      <c r="H27" t="s">
+        <v>23</v>
+      </c>
+      <c r="I27" t="s">
+        <v>128</v>
+      </c>
+      <c r="J27">
+        <v>0</v>
+      </c>
+      <c r="K27" t="s">
+        <v>43</v>
+      </c>
+      <c r="L27" t="s">
+        <v>66</v>
+      </c>
+      <c r="M27" t="s">
+        <v>26</v>
+      </c>
+      <c r="N27">
+        <v>1500</v>
+      </c>
+      <c r="O27" t="s">
+        <v>23</v>
+      </c>
+      <c r="P27">
+        <v>4</v>
+      </c>
+      <c r="Q27">
+        <v>6000</v>
+      </c>
+      <c r="R27" t="s">
+        <v>23</v>
+      </c>
+      <c r="S27" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>